<commit_message>
feat(tasks): AI bulk subtasks + status/progress palette + dark-mode polish
- New AI bulk subtasks screen (POST /tasks/{id}/subtasks/ai-bulk):
  semicolon-separated titles, smart defaults (progress, due-date mode),
  live `;` normalization, rate-limit countdown.
- Expandable FAB (Customize variant) on subtasks tab — RTL-aware.
- Status & progress color palette unified across slider, bar, and chips:
  red 0 → orange 1-69 → blue 70-99 → green 100, plus purple for HOLD.
- Parent-task lock: respects backend's `permissions.can_update_progress`,
  shows "computed from N subtasks" hint, maps PARENT_PROGRESS_LOCKED.
- Dark-mode fixes: parent/help/cooldown banners, mode chips, and
  OutlinedButton/TextButton foreground defaults to white.
- Date display via AppFuns.formatDate (Arabic locale, English digits).
- Hide keyboard on submit in AI screen + Add task screen.
- Cap AI input at 500 chars to conserve provider tokens.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/تطبيق موظفين نيوهورايزن.xlsx
+++ b/تطبيق موظفين نيوهورايزن.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mustapha\Documents\app_project\hr_portal\hr_portal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mustapha\Documents\GitHub\hrportal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8E8718-4F98-41E9-8FD8-566298955778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E0425F-9B28-4C96-9782-3FB57863AB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -602,7 +602,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -635,12 +635,6 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF1565C0"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
       <color rgb="FFC62828"/>
       <name val="Arial"/>
     </font>
@@ -657,7 +651,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -687,11 +681,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F5F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBBDEFB"/>
       </patternFill>
     </fill>
     <fill>
@@ -727,7 +716,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -756,18 +745,15 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2157,8 +2143,8 @@
       <c r="E47" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F47" s="9" t="s">
-        <v>129</v>
+      <c r="F47" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>151</v>
@@ -2272,8 +2258,8 @@
       <c r="E52" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F52" s="10" t="s">
-        <v>164</v>
+      <c r="F52" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="G52" s="8" t="s">
         <v>168</v>
@@ -2295,8 +2281,8 @@
       <c r="E53" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F53" s="10" t="s">
-        <v>164</v>
+      <c r="F53" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>171</v>
@@ -2318,7 +2304,7 @@
       <c r="E54" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F54" s="10" t="s">
+      <c r="F54" s="9" t="s">
         <v>164</v>
       </c>
       <c r="G54" s="8" t="s">
@@ -2341,7 +2327,7 @@
       <c r="E55" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F55" s="10" t="s">
+      <c r="F55" s="9" t="s">
         <v>164</v>
       </c>
       <c r="G55" s="5" t="s">
@@ -2349,118 +2335,118 @@
       </c>
     </row>
     <row r="57" spans="1:7" ht="16.899999999999999" x14ac:dyDescent="0.5">
-      <c r="A57" s="14" t="s">
+      <c r="A57" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="B57" s="13"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="13"/>
+      <c r="B57" s="12"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="C58" s="12" t="s">
+      <c r="C58" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B59" s="11" t="s">
+      <c r="B59" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C59" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
+      <c r="C59" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B60" s="11" t="s">
+      <c r="B60" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="C60" s="12" t="s">
+      <c r="C60" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="D60" s="13"/>
-      <c r="E60" s="13"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B61" s="11" t="s">
+      <c r="B61" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="C61" s="12" t="s">
+      <c r="C61" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="D61" s="13"/>
-      <c r="E61" s="13"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="12"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="C62" s="12" t="s">
+      <c r="C62" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="D62" s="13"/>
-      <c r="E62" s="13"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="12"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B63" s="11" t="s">
+      <c r="B63" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="C63" s="12" t="s">
+      <c r="C63" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="D63" s="13"/>
-      <c r="E63" s="13"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B64" s="11" t="s">
+      <c r="B64" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="C64" s="12" t="s">
+      <c r="C64" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="13"/>
+      <c r="D64" s="12"/>
+      <c r="E64" s="12"/>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B65" s="11" t="s">
+      <c r="B65" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="C65" s="12" t="s">
+      <c r="C65" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="D65" s="13"/>
-      <c r="E65" s="13"/>
+      <c r="D65" s="12"/>
+      <c r="E65" s="12"/>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B66" s="11" t="s">
+      <c r="B66" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="C66" s="12" t="s">
+      <c r="C66" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="D66" s="13"/>
-      <c r="E66" s="13"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C64:E64"/>
     <mergeCell ref="A57:G57"/>
     <mergeCell ref="C63:E63"/>
     <mergeCell ref="C62:E62"/>
     <mergeCell ref="C58:E58"/>
     <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C64:E64"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>